<commit_message>
scan: seg5 2026-08-28 18:32 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq6_2026-08-28.xlsx
+++ b/output/full_scan/batch_seq6_2026-08-28.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O83"/>
+  <dimension ref="A1:O84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -845,21 +845,21 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>6438</v>
+        <v>6225</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>迅得</t>
+          <t>天瀚</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v/>
       </c>
       <c r="D8" s="2" t="n">
-        <v>618.6067864313409</v>
+        <v>657.4762881015786</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>151</v>
+        <v>59.5</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -870,16 +870,16 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>57.19483006345361</v>
+        <v>67.42976435018691</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>14.25111738375986</v>
+        <v>51.8201513849315</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>2.327848704847906</v>
+        <v>1.078394137815737</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>0</v>
@@ -888,31 +888,31 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>0.9605244132881998</v>
+        <v>1.884597247182206</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>6284</v>
+        <v>6438</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>佳邦</t>
+          <t>迅得</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v/>
       </c>
       <c r="D9" s="2" t="n">
-        <v>608.0648281424041</v>
+        <v>618.6067864313409</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>81.40000000000001</v>
+        <v>151</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -923,16 +923,16 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>53.14340517031061</v>
+        <v>57.19483006345361</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>17.02257106718804</v>
+        <v>14.25111738375986</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>2.897662852765586</v>
+        <v>2.327848704847906</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>0</v>
@@ -941,31 +941,31 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>1.005026002669722</v>
+        <v>0.9605244132881998</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, liquidity_ok, obv_uptrend, dealer_buy_3d, bb_squeeze_breakout, cci_momentum, mfi_strong</t>
+          <t>volume_break, rsi_strong, breakout_20d, market_above_ma60, avoid_chase, obv_uptrend, breakout_volume_confirm, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>6290</v>
+        <v>6284</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>良維</t>
+          <t>佳邦</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v/>
       </c>
       <c r="D10" s="2" t="n">
-        <v>605.9113494879764</v>
+        <v>608.0648281424041</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>248</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -976,16 +976,16 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>57.82341983742649</v>
+        <v>53.14340517031061</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>25.26214737873338</v>
+        <v>17.02257106718804</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>1.191134948797634</v>
+        <v>2.897662852765586</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L10" s="2" t="n">
         <v>0</v>
@@ -994,31 +994,31 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>6.567802564555347</v>
+        <v>1.005026002669722</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, bb_squeeze_breakout, mfi_strong</t>
+          <t>volume_break, market_above_ma60, liquidity_ok, obv_uptrend, dealer_buy_3d, bb_squeeze_breakout, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>6426</v>
+        <v>6290</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>統新</t>
+          <t>良維</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v/>
       </c>
       <c r="D11" s="2" t="n">
-        <v>594.8068496958571</v>
+        <v>605.9113494879764</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>263.5</v>
+        <v>248</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>67.11578250326315</v>
+        <v>57.82341983742649</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>32.47468482274172</v>
+        <v>25.26214737873338</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>1.125632550007205</v>
+        <v>1.191134948797634</v>
       </c>
       <c r="K11" s="2" t="n">
         <v>0</v>
@@ -1047,31 +1047,31 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>4.055744527284368</v>
+        <v>6.567802564555347</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, bb_squeeze_breakout, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>6265</v>
+        <v>6426</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>方土昶</t>
+          <t>統新</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v/>
       </c>
       <c r="D12" s="2" t="n">
-        <v>579.9118456708223</v>
+        <v>594.8068496958571</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>57.1</v>
+        <v>263.5</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -1082,13 +1082,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>52.78109223899119</v>
+        <v>67.11578250326315</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>22.97010456817325</v>
+        <v>32.47468482274172</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>0.4528480115497993</v>
+        <v>1.125632550007205</v>
       </c>
       <c r="K12" s="2" t="n">
         <v>0</v>
@@ -1100,31 +1100,31 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>-0.18951666906253</v>
+        <v>4.055744527284368</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>6456</v>
+        <v>6265</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>GIS-KY</t>
+          <t>方土昶</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>570.542626497388</v>
+        <v>579.9118456708223</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>74.3</v>
+        <v>57.1</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -1135,13 +1135,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>61.74696784082273</v>
+        <v>52.78109223899119</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>15.35610190823388</v>
+        <v>22.97010456817325</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>2.564407789822586</v>
+        <v>0.4528480115497993</v>
       </c>
       <c r="K13" s="2" t="n">
         <v>0</v>
@@ -1153,31 +1153,31 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.976940995894704</v>
+        <v>-0.18951666906253</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>6435</v>
+        <v>6456</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>大中</t>
+          <t>GIS-KY</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v/>
       </c>
       <c r="D14" s="2" t="n">
-        <v>565.3622245638517</v>
+        <v>570.542626497388</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>260</v>
+        <v>74.3</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -1188,13 +1188,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>47.26400150798319</v>
+        <v>61.74696784082273</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>16.31567192982902</v>
+        <v>15.35610190823388</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>1.958185921330617</v>
+        <v>2.564407789822586</v>
       </c>
       <c r="K14" s="2" t="n">
         <v>0</v>
@@ -1206,31 +1206,31 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>2.914447824151116</v>
+        <v>0.976940995894704</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, obv_uptrend, breakout_volume_confirm, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>6263</v>
+        <v>6435</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>普萊德</t>
+          <t>大中</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v/>
       </c>
       <c r="D15" s="2" t="n">
-        <v>559.1726266424835</v>
+        <v>565.3622245638517</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>165.5</v>
+        <v>260</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1241,16 +1241,16 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>59.55245333029796</v>
+        <v>47.26400150798319</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>12.75215822364444</v>
+        <v>16.31567192982902</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>0.6794076078918447</v>
+        <v>1.958185921330617</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0</v>
@@ -1259,31 +1259,31 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.6400325968088065</v>
+        <v>2.914447824151116</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>6279</v>
+        <v>6263</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>胡連</t>
+          <t>普萊德</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v/>
       </c>
       <c r="D16" s="2" t="n">
-        <v>558.2339961290573</v>
+        <v>559.1726266424835</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>127</v>
+        <v>165.5</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1294,16 +1294,16 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>57.36330552587825</v>
+        <v>59.55245333029796</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>15.99076948518842</v>
+        <v>12.75215822364444</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>0.6218522680812315</v>
+        <v>0.6794076078918447</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0</v>
@@ -1312,31 +1312,31 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>-0.2363843412215835</v>
+        <v>0.6400325968088065</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>6237</v>
+        <v>6279</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>驊訊</t>
+          <t>胡連</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v/>
       </c>
       <c r="D17" s="2" t="n">
-        <v>553.1624981558506</v>
+        <v>558.2339961290573</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>35.2</v>
+        <v>127</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1347,16 +1347,16 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>50.99360438501209</v>
+        <v>57.36330552587825</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>22.44276380005408</v>
+        <v>15.99076948518842</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>1.097505839344393</v>
+        <v>0.6218522680812315</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0</v>
@@ -1365,31 +1365,31 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.4507018063713963</v>
+        <v>-0.2363843412215835</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>6175</v>
+        <v>6237</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>立敦</t>
+          <t>驊訊</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
         <v/>
       </c>
       <c r="D18" s="2" t="n">
-        <v>550.9029365627376</v>
+        <v>553.1624981558506</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>76.8</v>
+        <v>35.2</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1400,16 +1400,16 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>46.5339987911337</v>
+        <v>50.99360438501209</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>19.13504901359752</v>
+        <v>22.44276380005408</v>
       </c>
       <c r="J18" s="2" t="n">
-        <v>1.904619479937037</v>
+        <v>1.097505839344393</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L18" s="2" t="n">
         <v>0</v>
@@ -1418,31 +1418,31 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>0.8118251722129326</v>
+        <v>0.4507018063713963</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>6446</v>
+        <v>6175</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>藥華藥</t>
+          <t>立敦</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>535.8010776393595</v>
+        <v>550.9029365627376</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1545</v>
+        <v>76.8</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1453,13 +1453,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>64.19129235367168</v>
+        <v>46.5339987911337</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>36.97204546865093</v>
+        <v>19.13504901359752</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>1.023326416480007</v>
+        <v>1.904619479937037</v>
       </c>
       <c r="K19" s="2" t="n">
         <v>0</v>
@@ -1471,31 +1471,31 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>12.65351345053263</v>
+        <v>0.8118251722129326</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>6472</v>
+        <v>6446</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>保瑞</t>
+          <t>藥華藥</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>520.9712675240604</v>
+        <v>535.8010776393595</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>435</v>
+        <v>1545</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1506,13 +1506,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>53.23162666339669</v>
+        <v>64.19129235367168</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>30.01872851240987</v>
+        <v>36.97204546865093</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>0.6774247421735233</v>
+        <v>1.023326416480007</v>
       </c>
       <c r="K20" s="2" t="n">
         <v>0</v>
@@ -1524,31 +1524,31 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>2.153630574639546</v>
+        <v>12.65351345053263</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>6173</v>
+        <v>6472</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>信昌電</t>
+          <t>保瑞</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v/>
       </c>
       <c r="D21" s="2" t="n">
-        <v>515.6244352996924</v>
+        <v>520.9712675240604</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>239</v>
+        <v>435</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1559,16 +1559,16 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>60.62088414880052</v>
+        <v>53.23162666339669</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>18.4490954828624</v>
+        <v>30.01872851240987</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>1.236559362589119</v>
+        <v>0.6774247421735233</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L21" s="2" t="n">
         <v>0</v>
@@ -1577,31 +1577,31 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>5.288093809646383</v>
+        <v>2.153630574639546</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>6419</v>
+        <v>6173</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>京晨科</t>
+          <t>信昌電</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v/>
       </c>
       <c r="D22" s="2" t="n">
-        <v>511.7346347621678</v>
+        <v>515.6244352996924</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>154</v>
+        <v>239</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1612,16 +1612,16 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>52.10969393183165</v>
+        <v>60.62088414880052</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>22.96352159268069</v>
+        <v>18.4490954828624</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>0.5543557108942232</v>
+        <v>1.236559362589119</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L22" s="2" t="n">
         <v>0</v>
@@ -1630,31 +1630,31 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>-1.003678473111092</v>
+        <v>5.288093809646383</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>6170</v>
+        <v>6419</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>統振</t>
+          <t>京晨科</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
         <v/>
       </c>
       <c r="D23" s="2" t="n">
-        <v>510.9737452021472</v>
+        <v>511.7346347621678</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>48.7</v>
+        <v>154</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -1665,16 +1665,16 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>59.87316342198224</v>
+        <v>52.10969393183165</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>22.62973438293024</v>
+        <v>22.96352159268069</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>1.328419899795577</v>
+        <v>0.5543557108942232</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L23" s="2" t="n">
         <v>0</v>
@@ -1683,31 +1683,31 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.3071501608575315</v>
+        <v>-1.003678473111092</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>6416</v>
+        <v>6170</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>瑞祺電通</t>
+          <t>統振</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>507.2306052356462</v>
+        <v>510.9737452021472</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>100.5</v>
+        <v>48.7</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,16 +1718,16 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>54.68491343423481</v>
+        <v>59.87316342198224</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>15.18679627488019</v>
+        <v>22.62973438293024</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.7120825074308554</v>
+        <v>1.328419899795577</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>0</v>
@@ -1736,31 +1736,31 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.0370771972821259</v>
+        <v>0.3071501608575315</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>6174</v>
+        <v>6416</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>安碁</t>
+          <t>瑞祺電通</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>502.0400247298541</v>
+        <v>507.2306052356462</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>45.55</v>
+        <v>100.5</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,16 +1771,16 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>51.25242209637744</v>
+        <v>54.68491343423481</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>13.14254361812471</v>
+        <v>15.18679627488019</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.4193879097243387</v>
+        <v>0.7120825074308554</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>0.5021054851771137</v>
+        <v>0.0370771972821259</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>6291</v>
+        <v>6174</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>沛亨</t>
+          <t>安碁</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>494.7742902676001</v>
+        <v>502.0400247298541</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>400.5</v>
+        <v>45.55</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,16 +1824,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>51.85003065508189</v>
+        <v>51.25242209637744</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>16.63492481856979</v>
+        <v>13.14254361812471</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>2.072095663081945</v>
+        <v>0.4193879097243387</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>7.287706320092807</v>
+        <v>0.5021054851771137</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6259</v>
+        <v>6291</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>百徽</t>
+          <t>沛亨</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>477.4396460159516</v>
+        <v>494.7742902676001</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>31.75</v>
+        <v>400.5</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,16 +1877,16 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>52.56306860794313</v>
+        <v>51.85003065508189</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>10.62582170750973</v>
+        <v>16.63492481856979</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>1.446261807903215</v>
+        <v>2.072095663081945</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.1446846854098987</v>
+        <v>7.287706320092807</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, foreign_buy_3d, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>6207</v>
+        <v>6259</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>雷科</t>
+          <t>百徽</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>475.2675656740154</v>
+        <v>477.4396460159516</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>111</v>
+        <v>31.75</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,16 +1930,16 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>51.94776785096845</v>
+        <v>52.56306860794313</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>14.0112972316025</v>
+        <v>10.62582170750973</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>1.559500269989604</v>
+        <v>1.446261807903215</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L28" s="2" t="n">
         <v>0</v>
@@ -1948,31 +1948,31 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1.677214377350343</v>
+        <v>0.1446846854098987</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, foreign_buy_3d, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6423</v>
+        <v>6207</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>億而得-創</t>
+          <t>雷科</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>474.3245576878028</v>
+        <v>475.2675656740154</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>80.90000000000001</v>
+        <v>111</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,16 +1983,16 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>56.58319715958275</v>
+        <v>51.94776785096845</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>15.88745882328509</v>
+        <v>14.0112972316025</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.4078120710478514</v>
+        <v>1.559500269989604</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="L29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.3414882727416246</v>
+        <v>1.677214377350343</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, obv_uptrend, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>6204</v>
+        <v>6423</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>艾華</t>
+          <t>億而得-創</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>462.1224552186068</v>
+        <v>474.3245576878028</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>88.40000000000001</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,16 +2036,16 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>57.02079273045774</v>
+        <v>56.58319715958275</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>18.43084671172283</v>
+        <v>15.88745882328509</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>3.044500897357133</v>
+        <v>0.4078120710478514</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="L30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>1.44224527028846</v>
+        <v>0.3414882727416246</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, cci_momentum, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6449</v>
+        <v>6204</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>鈺邦</t>
+          <t>艾華</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>460.6618748371263</v>
+        <v>462.1224552186068</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>237</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,13 +2089,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>49.38887030804914</v>
+        <v>57.02079273045774</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>24.58315881884735</v>
+        <v>18.43084671172283</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>3.511025486023218</v>
+        <v>3.044500897357133</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>3.689088689701862</v>
+        <v>1.44224527028846</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, rsi_strong, market_above_ma60, avoid_chase, cci_momentum, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6185</v>
+        <v>6449</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>幃翔</t>
+          <t>鈺邦</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>434.6997843927652</v>
+        <v>460.6618748371263</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>12.65</v>
+        <v>237</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,16 +2142,16 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>29.77127464225732</v>
+        <v>49.38887030804914</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>25.64379000446028</v>
+        <v>24.58315881884735</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.6182511143073882</v>
+        <v>3.511025486023218</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.0662192697496226</v>
+        <v>3.689088689701862</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>6210</v>
+        <v>6185</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>慶生</t>
+          <t>幃翔</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>430.4953875249219</v>
+        <v>434.6997843927652</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>18.05</v>
+        <v>12.65</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,16 +2195,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>51.5932367200336</v>
+        <v>29.77127464225732</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>6.725795539635822</v>
+        <v>25.64379000446028</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.1085244745973179</v>
+        <v>0.6182511143073882</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.1379442792191344</v>
+        <v>-0.0662192697496226</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>6220</v>
+        <v>6210</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>岳豐</t>
+          <t>慶生</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>428.9261518403976</v>
+        <v>430.4953875249219</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>25.9</v>
+        <v>18.05</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,16 +2248,16 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>42.47451663847761</v>
+        <v>51.5932367200336</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>22.38136071901567</v>
+        <v>6.725795539635822</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>1.184980529164982</v>
+        <v>0.1085244745973179</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.3039984578961547</v>
+        <v>0.1379442792191344</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, cci_momentum, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>6415</v>
+        <v>6220</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>矽力*-KY</t>
+          <t>岳豐</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>427.6799074905534</v>
+        <v>428.9261518403976</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>458</v>
+        <v>25.9</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,16 +2301,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>49.15178573589615</v>
+        <v>42.47451663847761</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>11.31310597754299</v>
+        <v>22.38136071901567</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>1.378073766106229</v>
+        <v>1.184980529164982</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>4.752995185122723</v>
+        <v>0.3039984578961547</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>6208</v>
+        <v>6415</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>日揚</t>
+          <t>矽力*-KY</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>424.4245981761354</v>
+        <v>427.6799074905534</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>82.7</v>
+        <v>458</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,16 +2354,16 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>49.16256896810333</v>
+        <v>49.15178573589615</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>9.036185608400103</v>
+        <v>11.31310597754299</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>0.6379396716921866</v>
+        <v>1.378073766106229</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.4009681186222096</v>
+        <v>4.752995185122723</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>6464</v>
+        <v>6208</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>台數科</t>
+          <t>日揚</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>421.1628433975877</v>
+        <v>424.4245981761354</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>77.40000000000001</v>
+        <v>82.7</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,16 +2407,16 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>43.23754751029882</v>
+        <v>49.16256896810333</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>30.3614898747337</v>
+        <v>9.036185608400103</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.0264456456029753</v>
+        <v>0.6379396716921866</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L37" s="2" t="n">
         <v>0</v>
@@ -2425,31 +2425,31 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.0482342125525407</v>
+        <v>0.4009681186222096</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>6462</v>
+        <v>6464</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>神盾</t>
+          <t>台數科</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>420.5907742526043</v>
+        <v>421.1628433975877</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>101</v>
+        <v>77.40000000000001</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,16 +2460,16 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>50.89135720946131</v>
+        <v>43.23754751029882</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>12.23656176637316</v>
+        <v>30.3614898747337</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>1.209885155478894</v>
+        <v>0.0264456456029753</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L38" s="2" t="n">
         <v>0</v>
@@ -2478,31 +2478,31 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.6630354197146278</v>
+        <v>-0.0482342125525407</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6474</v>
+        <v>6462</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>華豫寧</t>
+          <t>神盾</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>417.4166039771195</v>
+        <v>420.5907742526043</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>37.2</v>
+        <v>101</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,16 +2513,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>42.94906914469832</v>
+        <v>50.89135720946131</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>14.52416864362302</v>
+        <v>12.23656176637316</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>1.34166039771195</v>
+        <v>1.209885155478894</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-0.1306484979613549</v>
+        <v>0.6630354197146278</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>6241</v>
+        <v>6474</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>鑫永洋</t>
+          <t>華豫寧</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>414.5609851099871</v>
+        <v>417.4166039771195</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>17.95</v>
+        <v>37.2</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,13 +2566,13 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>64.24087223278788</v>
+        <v>42.94906914469832</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>23.75233044816658</v>
+        <v>14.52416864362302</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.5703510131950319</v>
+        <v>1.34166039771195</v>
       </c>
       <c r="K40" s="2" t="n">
         <v>0</v>
@@ -2584,31 +2584,31 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>0.2491523504345987</v>
+        <v>-0.1306484979613549</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6274</v>
+        <v>6241</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>台燿</t>
+          <t>鑫永洋</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>412.270691863583</v>
+        <v>414.5609851099871</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>1490</v>
+        <v>17.95</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,16 +2619,16 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>51.12197071468819</v>
+        <v>64.24087223278788</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>12.92753830817594</v>
+        <v>23.75233044816658</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.9268584740680228</v>
+        <v>0.5703510131950319</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
         <v>0</v>
@@ -2637,31 +2637,31 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-6.403204721060959</v>
+        <v>0.2491523504345987</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, rsi_strong, breakout_20d, market_above_ma60, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>6234</v>
+        <v>6274</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>高僑</t>
+          <t>台燿</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>409.4035175615221</v>
+        <v>412.270691863583</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>36.8</v>
+        <v>1490</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,16 +2672,16 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>50.97575090432648</v>
+        <v>51.12197071468819</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>19.28136961737346</v>
+        <v>12.92753830817594</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>1.064029708868585</v>
+        <v>0.9268584740680228</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L42" s="2" t="n">
         <v>0</v>
@@ -2690,31 +2690,31 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>0.4117766085772416</v>
+        <v>-6.403204721060959</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>6163</v>
+        <v>6234</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>華電網</t>
+          <t>高僑</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>393.8380620056482</v>
+        <v>409.4035175615221</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>43.3</v>
+        <v>36.8</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,16 +2725,16 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>51.83257002002662</v>
+        <v>50.97575090432648</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>16.58435840139506</v>
+        <v>19.28136961737346</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.3501319006439303</v>
+        <v>1.064029708868585</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.2866547032570856</v>
+        <v>0.4117766085772416</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>6227</v>
+        <v>6163</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>茂綸</t>
+          <t>華電網</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>391.9745330145391</v>
+        <v>393.8380620056482</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>113</v>
+        <v>43.3</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>42.62766745040317</v>
+        <v>51.83257002002662</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>10.53080062410892</v>
+        <v>16.58435840139506</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>4.054870709294181</v>
+        <v>0.3501319006439303</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.6635121858485432</v>
+        <v>0.2866547032570856</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6442</v>
+        <v>6227</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>茂綸</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>384.5979482790846</v>
+        <v>391.9745330145391</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1615</v>
+        <v>113</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,13 +2831,13 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>57.24637714399277</v>
+        <v>42.62766745040317</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>19.95431833788605</v>
+        <v>10.53080062410892</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.493409533669333</v>
+        <v>4.054870709294181</v>
       </c>
       <c r="K45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>17.52843645163279</v>
+        <v>-0.6635121858485432</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6229</v>
+        <v>6442</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>研通</t>
+          <t>光聖</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>383.3000374553882</v>
+        <v>384.5979482790846</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>24.1</v>
+        <v>1615</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>52.34524013146724</v>
+        <v>57.24637714399277</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>13.68205950377573</v>
+        <v>19.95431833788605</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>1.762612414550255</v>
+        <v>0.493409533669333</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.0991587690144452</v>
+        <v>17.52843645163279</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>rsi_strong, market_above_ma60, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>6412</v>
+        <v>6229</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>群電</t>
+          <t>研通</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>376.360288894505</v>
+        <v>383.3000374553882</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>79.09999999999999</v>
+        <v>24.1</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,16 +2937,16 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>47.21767055504127</v>
+        <v>52.34524013146724</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>25.10644298527706</v>
+        <v>13.68205950377573</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>0.7415293581518918</v>
+        <v>1.762612414550255</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.443540842323328</v>
+        <v>0.0991587690144452</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6184</v>
+        <v>6412</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>大豐電</t>
+          <t>群電</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>371.1568356212218</v>
+        <v>376.360288894505</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>41.15</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>21.62858491618736</v>
+        <v>47.21767055504127</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>24.10473848119856</v>
+        <v>25.10644298527706</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>2.018218801074867</v>
+        <v>0.7415293581518918</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.006847004746841</v>
+        <v>0.443540842323328</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>6270</v>
+        <v>6184</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>倍微</t>
+          <t>大豐電</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>367.8605009579209</v>
+        <v>371.1568356212218</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>29.95</v>
+        <v>41.15</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>47.40322508293248</v>
+        <v>21.62858491618736</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>9.46827354533465</v>
+        <v>24.10473848119856</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.7889084630381776</v>
+        <v>2.018218801074867</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.132156110709524</v>
+        <v>-0.006847004746841</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>6244</v>
+        <v>6270</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>茂迪</t>
+          <t>倍微</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>366.0008243905912</v>
+        <v>367.8605009579209</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>24.4</v>
+        <v>29.95</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>47.43175601889502</v>
+        <v>47.40322508293248</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>16.7927897377716</v>
+        <v>9.46827354533465</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.8132732249174556</v>
+        <v>0.7889084630381776</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>0.0455341167057048</v>
+        <v>0.132156110709524</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6409</v>
+        <v>6244</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>旭隼</t>
+          <t>茂迪</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>359.4423663389936</v>
+        <v>366.0008243905912</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>1030</v>
+        <v>24.4</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,16 +3149,16 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>53.00282509475455</v>
+        <v>47.43175601889502</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>19.82458603953884</v>
+        <v>16.7927897377716</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.9133591150753484</v>
+        <v>0.8132732249174556</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>2.908216477448301</v>
+        <v>0.0455341167057048</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>6470</v>
+        <v>6409</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>宇智</t>
+          <t>旭隼</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>359.4104136311823</v>
+        <v>359.4423663389936</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>41.5</v>
+        <v>1030</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,16 +3202,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>30.03800412225367</v>
+        <v>53.00282509475455</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>44.49327720108618</v>
+        <v>19.82458603953884</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>1.838312980571893</v>
+        <v>0.9133591150753484</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>0.1677168333790377</v>
+        <v>2.908216477448301</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6275</v>
+        <v>6470</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>元山</t>
+          <t>宇智</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>355.5467219852067</v>
+        <v>359.4104136311823</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>45.7</v>
+        <v>41.5</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>54.84932866837448</v>
+        <v>30.03800412225367</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>20.7208457549255</v>
+        <v>44.49327720108618</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.9285922868864732</v>
+        <v>1.838312980571893</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.3662160488750076</v>
+        <v>0.1677168333790377</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6441</v>
+        <v>6275</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>廣錠</t>
+          <t>元山</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>354.7319013947222</v>
+        <v>355.5467219852067</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>21.25</v>
+        <v>45.7</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>46.35393956337096</v>
+        <v>54.84932866837448</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>20.79559484497857</v>
+        <v>20.7208457549255</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.2287842697406492</v>
+        <v>0.9285922868864732</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-0.0455670878242028</v>
+        <v>0.3662160488750076</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>6223</v>
+        <v>6441</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>旺矽</t>
+          <t>廣錠</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>352.0178342813626</v>
+        <v>354.7319013947222</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>5030</v>
+        <v>21.25</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>38.99996869182381</v>
+        <v>46.35393956337096</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>17.49696131085538</v>
+        <v>20.79559484497857</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>1.720442525144879</v>
+        <v>0.2287842697406492</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-87.89762703964971</v>
+        <v>-0.0455670878242028</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6177</v>
+        <v>6223</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>達麗</t>
+          <t>旺矽</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>348.0789735296511</v>
+        <v>352.0178342813626</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>47.55</v>
+        <v>5030</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>48.98412584385693</v>
+        <v>38.99996869182381</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>22.30949566943033</v>
+        <v>17.49696131085538</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.5017343842174131</v>
+        <v>1.720442525144879</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.0896014490521822</v>
+        <v>-87.89762703964971</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6477</v>
+        <v>6177</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>安集</t>
+          <t>達麗</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>347.1079109224706</v>
+        <v>348.0789735296511</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>37.05</v>
+        <v>47.55</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>51.52182334116729</v>
+        <v>48.98412584385693</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>19.29824582664845</v>
+        <v>22.30949566943033</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.93870330744171</v>
+        <v>0.5017343842174131</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.0820561911325131</v>
+        <v>-0.0896014490521822</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6261</v>
+        <v>6477</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>久元</t>
+          <t>安集</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>346.6161974133568</v>
+        <v>347.1079109224706</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>79</v>
+        <v>37.05</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,16 +3520,16 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>46.61462627794441</v>
+        <v>51.52182334116729</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>24.11080892504607</v>
+        <v>19.29824582664845</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.599697291418178</v>
+        <v>0.93870330744171</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.8251722097627407</v>
+        <v>0.0820561911325131</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>6285</v>
+        <v>6261</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>啟碁</t>
+          <t>久元</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>342.1137505009763</v>
+        <v>346.6161974133568</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>247</v>
+        <v>79</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,16 +3573,16 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>52.5117609128559</v>
+        <v>46.61462627794441</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>14.65286880017313</v>
+        <v>24.11080892504607</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.8739918625535201</v>
+        <v>0.599697291418178</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.9593927139235769</v>
+        <v>0.8251722097627407</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>6182</v>
+        <v>6285</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>合晶</t>
+          <t>啟碁</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>338.6366182498644</v>
+        <v>342.1137505009763</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>110</v>
+        <v>247</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>49.13765272743972</v>
+        <v>52.5117609128559</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>12.81016665108128</v>
+        <v>14.65286880017313</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1.213413776033681</v>
+        <v>0.8739918625535201</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>0.9265515078521238</v>
+        <v>0.9593927139235769</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6405</v>
+        <v>6182</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>悅城</t>
+          <t>合晶</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>333.3338712222049</v>
+        <v>338.6366182498644</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>40.25</v>
+        <v>110</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>46.72265707437822</v>
+        <v>49.13765272743972</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>24.54390258398169</v>
+        <v>12.81016665108128</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.7389387444466331</v>
+        <v>1.213413776033681</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.8259068597699337</v>
+        <v>0.9265515078521238</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6432</v>
+        <v>6405</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>今展科</t>
+          <t>悅城</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>323.5462144049748</v>
+        <v>333.3338712222049</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>65.40000000000001</v>
+        <v>40.25</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,13 +3732,13 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>43.45570214660007</v>
+        <v>46.72265707437822</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>13.19116676537168</v>
+        <v>24.54390258398169</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.6213561482179417</v>
+        <v>0.7389387444466331</v>
       </c>
       <c r="K62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.7211590378078467</v>
+        <v>0.8259068597699337</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>6194</v>
+        <v>6432</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>育富</t>
+          <t>今展科</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>322.5908232948232</v>
+        <v>323.5462144049748</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>29.75</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>45.21827202448242</v>
+        <v>43.45570214660007</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>23.30738593648126</v>
+        <v>13.19116676537168</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>0.1230707791896783</v>
+        <v>0.6213561482179417</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.0918261252179387</v>
+        <v>-0.7211590378078467</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>6217</v>
+        <v>6194</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>中探針</t>
+          <t>育富</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>314.5316449997685</v>
+        <v>322.5908232948232</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>175</v>
+        <v>29.75</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,16 +3838,16 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>54.40506400943818</v>
+        <v>45.21827202448242</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>14.31692475889225</v>
+        <v>23.30738593648126</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>4.33486317435983</v>
+        <v>0.1230707791896783</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L64" s="2" t="n">
         <v>0</v>
@@ -3856,31 +3856,31 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>5.036421131024584</v>
+        <v>0.0918261252179387</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>6167</v>
+        <v>6217</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>久正</t>
+          <t>中探針</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>307.3855596769686</v>
+        <v>314.5316449997685</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>10.8</v>
+        <v>175</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,13 +3891,13 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>51.93181629537075</v>
+        <v>54.40506400943818</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>14.24282284221066</v>
+        <v>14.31692475889225</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>1.90282628172046</v>
+        <v>4.33486317435983</v>
       </c>
       <c r="K65" s="2" t="n">
         <v>0</v>
@@ -3909,31 +3909,31 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.0809255956632683</v>
+        <v>5.036421131024584</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend, dealer_buy_3d</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>6411</v>
+        <v>6167</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>晶焱</t>
+          <t>久正</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>303.5091746935789</v>
+        <v>307.3855596769686</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>80.09999999999999</v>
+        <v>10.8</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>50.09104576974312</v>
+        <v>51.93181629537075</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>14.83096258585797</v>
+        <v>14.24282284221066</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.8576720603347204</v>
+        <v>1.90282628172046</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.7924503329776313</v>
+        <v>0.0809255956632683</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend, dealer_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>6266</v>
+        <v>6411</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>泰詠</t>
+          <t>晶焱</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>300.6321083486163</v>
+        <v>303.5091746935789</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>25</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>49.37700214538894</v>
+        <v>50.09104576974312</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>11.33527041754093</v>
+        <v>14.83096258585797</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>1.013325201321883</v>
+        <v>0.8576720603347204</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>0.0514124334544068</v>
+        <v>0.7924503329776313</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4025,21 +4025,21 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>6233</v>
+        <v>6266</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>旺玖</t>
+          <t>泰詠</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>297.0458991394158</v>
+        <v>300.6321083486163</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>21.8</v>
+        <v>25</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>50.97364237328794</v>
+        <v>49.37700214538894</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>15.08153097060021</v>
+        <v>11.33527041754093</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.7111792673913935</v>
+        <v>1.013325201321883</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>0.1731308787126361</v>
+        <v>0.0514124334544068</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4078,21 +4078,21 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6198</v>
+        <v>6233</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>瑞築</t>
+          <t>旺玖</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>288.4497852454349</v>
+        <v>297.0458991394158</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>19.4</v>
+        <v>21.8</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>51.37019903168825</v>
+        <v>50.97364237328794</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>5.795319858454928</v>
+        <v>15.08153097060021</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.2859652996995775</v>
+        <v>0.7111792673913935</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.162056472757117</v>
+        <v>0.1731308787126361</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6236</v>
+        <v>6198</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>中湛</t>
+          <t>瑞築</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>283.6617050652613</v>
+        <v>288.4497852454349</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0</v>
+        <v>19.4</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,16 +4156,16 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>47.2661279169273</v>
+        <v>51.37019903168825</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>9.976568976137196</v>
+        <v>5.795319858454928</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0</v>
+        <v>0.2859652996995775</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.2234751754226422</v>
+        <v>0.162056472757117</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6451</v>
+        <v>6236</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>訊芯-KY</t>
+          <t>中湛</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>279.794120283499</v>
+        <v>283.6617050652613</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>453.5</v>
+        <v>0</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>52.91579407596211</v>
+        <v>47.2661279169273</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>10.69752315441651</v>
+        <v>9.976568976137196</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>1.234114533486751</v>
+        <v>0</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,51 +4227,51 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>6.255058280117531</v>
+        <v>0.2234751754226422</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6288</v>
+        <v>6451</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>聯嘉</t>
+          <t>訊芯-KY</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>274.1623227954031</v>
+        <v>279.794120283499</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>20.95</v>
+        <v>453.5</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2025-08-04</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="G72" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>45.12010230369736</v>
+        <v>52.91579407596211</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v/>
+        <v>10.69752315441651</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.6831032524092705</v>
+        <v>1.234114533486751</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>0</v>
@@ -4280,51 +4280,51 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0137243745044277</v>
+        <v>6.255058280117531</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6414</v>
+        <v>6288</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>樺漢</t>
+          <t>聯嘉</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>264.0002721951551</v>
+        <v>274.1623227954031</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>390</v>
+        <v>20.95</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2025-08-04</t>
         </is>
       </c>
       <c r="G73" s="2" t="b">
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>41.68839979028543</v>
+        <v>45.12010230369736</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>18.4106716409476</v>
+        <v/>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.4560360981553977</v>
+        <v>0.6831032524092705</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-5.616624631806086</v>
+        <v>0.0137243745044277</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6417</v>
+        <v>6414</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>韋僑</t>
+          <t>樺漢</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>263.0502509771013</v>
+        <v>264.0002721951551</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>106</v>
+        <v>390</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>36.25788448581032</v>
+        <v>41.68839979028543</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>25.06731680536659</v>
+        <v>18.4106716409476</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.4860053056529334</v>
+        <v>0.4560360981553977</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.1162007515605383</v>
+        <v>-5.616624631806086</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6283</v>
+        <v>6417</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>淳安</t>
+          <t>韋僑</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>258.9769870105815</v>
+        <v>263.0502509771013</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>20</v>
+        <v>106</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>41.04361467917883</v>
+        <v>36.25788448581032</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>30.73239472754121</v>
+        <v>25.06731680536659</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.7993180288706967</v>
+        <v>0.4860053056529334</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.0971779482326786</v>
+        <v>0.1162007515605383</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6245</v>
+        <v>6283</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>立端</t>
+          <t>淳安</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>254.5299629977683</v>
+        <v>258.9769870105815</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>83.2</v>
+        <v>20</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>51.64279509996974</v>
+        <v>41.04361467917883</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>11.27973762696614</v>
+        <v>30.73239472754121</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.8440487803055989</v>
+        <v>0.7993180288706967</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.1500699578030893</v>
+        <v>0.0971779482326786</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6276</v>
+        <v>6245</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>安鈦克</t>
+          <t>立端</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>250.6624404691856</v>
+        <v>254.5299629977683</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>20.25</v>
+        <v>83.2</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>50.01658479242569</v>
+        <v>51.64279509996974</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>22.49175526444076</v>
+        <v>11.27973762696614</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>1.122719002771823</v>
+        <v>0.8440487803055989</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.2275014374274705</v>
+        <v>-0.1500699578030893</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6246</v>
+        <v>6276</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>臺龍</t>
+          <t>安鈦克</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>249.6520045124877</v>
+        <v>250.6624404691856</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>12.25</v>
+        <v>20.25</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>41.68750515171868</v>
+        <v>50.01658479242569</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>20.73803786984623</v>
+        <v>22.49175526444076</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.2983311302048909</v>
+        <v>1.122719002771823</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.087105725225745</v>
+        <v>0.2275014374274705</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6443</v>
+        <v>6246</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>元晶</t>
+          <t>臺龍</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>231.263796666794</v>
+        <v>249.6520045124877</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>26.65</v>
+        <v>12.25</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,13 +4633,13 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>45.86875087372697</v>
+        <v>41.68750515171868</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>13.22248963298686</v>
+        <v>20.73803786984623</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>1.222973149677565</v>
+        <v>0.2983311302048909</v>
       </c>
       <c r="K79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.2854786076686182</v>
+        <v>0.087105725225745</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6222</v>
+        <v>6443</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>立軒</t>
+          <t>元晶</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>209.2952005868291</v>
+        <v>231.263796666794</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>20.05</v>
+        <v>26.65</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,13 +4686,13 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>51.33754290463593</v>
+        <v>45.86875087372697</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>9.04375991103098</v>
+        <v>13.22248963298686</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.3632252586844889</v>
+        <v>1.222973149677565</v>
       </c>
       <c r="K80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.3958481005208724</v>
+        <v>0.2854786076686182</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6228</v>
+        <v>6222</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>全譜</t>
+          <t>立軒</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>167.3930883486433</v>
+        <v>209.2952005868291</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>0</v>
+        <v>20.05</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,13 +4739,13 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>39.24634457150348</v>
+        <v>51.33754290463593</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>7.793237500110434</v>
+        <v>9.04375991103098</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.0115692307692307</v>
+        <v>0.3632252586844889</v>
       </c>
       <c r="K81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.5313049805255357</v>
+        <v>0.3958481005208724</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6188</v>
+        <v>6228</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>廣明</t>
+          <t>全譜</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>110.3490826174812</v>
+        <v>167.3930883486433</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>68.8</v>
+        <v>0</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>43.93803173043239</v>
+        <v>39.24634457150348</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>18.60514702148712</v>
+        <v>7.793237500110434</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.6140222457569217</v>
+        <v>0.0115692307692307</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.1391087176259233</v>
+        <v>-0.5313049805255357</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4820,52 +4820,105 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
+        <v>6188</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>廣明</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>110.3490826174812</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H83" s="2" t="n">
+        <v>43.93803173043239</v>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>18.60514702148712</v>
+      </c>
+      <c r="J83" s="2" t="n">
+        <v>0.6140222457569217</v>
+      </c>
+      <c r="K83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N83" s="2" t="n">
+        <v>0.1391087176259233</v>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
         <v>6203</v>
       </c>
-      <c r="B83" s="2" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>海韻電</t>
         </is>
       </c>
-      <c r="C83" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D83" s="2" t="n">
+      <c r="C84" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D84" s="2" t="n">
         <v>79.69256883947179</v>
       </c>
-      <c r="E83" s="2" t="n">
+      <c r="E84" s="2" t="n">
         <v>59.6</v>
       </c>
-      <c r="F83" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
-      </c>
-      <c r="G83" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H83" s="2" t="n">
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H84" s="2" t="n">
         <v>30.58572186742816</v>
       </c>
-      <c r="I83" s="2" t="n">
+      <c r="I84" s="2" t="n">
         <v>17.3651698807019</v>
       </c>
-      <c r="J83" s="2" t="n">
+      <c r="J84" s="2" t="n">
         <v>0.5193246202755211</v>
       </c>
-      <c r="K83" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L83" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M83" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N83" s="2" t="n">
+      <c r="K84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N84" s="2" t="n">
         <v>0.1237877631542381</v>
       </c>
-      <c r="O83" s="2" t="inlineStr">
+      <c r="O84" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>